<commit_message>
checkpoint: current progress before fixing comprehension saving issue
</commit_message>
<xml_diff>
--- a/mobile/ipa.xlsx
+++ b/mobile/ipa.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D197"/>
+  <dimension ref="A1:D376"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3157,9 +3157,2515 @@
         <v>by or from you</v>
       </c>
     </row>
+    <row r="198">
+      <c r="A198" t="str">
+        <v>adds</v>
+      </c>
+      <c r="B198" t="str">
+        <v>/ˈad/</v>
+      </c>
+      <c r="C198" t="str">
+        <v>to combine numbers into a single sum</v>
+      </c>
+      <c r="D198" t="str">
+        <v>to join or unite to something</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="str">
+        <v>all</v>
+      </c>
+      <c r="B199" t="str">
+        <v>/ˈȯl/</v>
+      </c>
+      <c r="C199" t="str">
+        <v>every one of</v>
+      </c>
+      <c r="D199" t="str">
+        <v>the whole of</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="str">
+        <v>ana</v>
+      </c>
+      <c r="B200" t="str">
+        <v/>
+      </c>
+      <c r="C200" t="str">
+        <v/>
+      </c>
+      <c r="D200" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="str">
+        <v>answered</v>
+      </c>
+      <c r="B201" t="str">
+        <v/>
+      </c>
+      <c r="C201" t="str">
+        <v>to speak or write in order to satisfy a question</v>
+      </c>
+      <c r="D201" t="str">
+        <v>to write a response to a letter or e-mail</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="str">
+        <v>anymore</v>
+      </c>
+      <c r="B202" t="str">
+        <v>/ˌe-nē-ˈmȯr/</v>
+      </c>
+      <c r="C202" t="str">
+        <v>in the recent or present period of time</v>
+      </c>
+      <c r="D202" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="str">
+        <v>around</v>
+      </c>
+      <c r="B203" t="str">
+        <v>/ə-ˈrau̇nd/</v>
+      </c>
+      <c r="C203" t="str">
+        <v>in circumference</v>
+      </c>
+      <c r="D203" t="str">
+        <v>in or along a curving course</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="str">
+        <v>asked</v>
+      </c>
+      <c r="B204" t="str">
+        <v>/ˈask/</v>
+      </c>
+      <c r="C204" t="str">
+        <v>to seek information by posing a question</v>
+      </c>
+      <c r="D204" t="str">
+        <v>to make a request</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="str">
+        <v>asks</v>
+      </c>
+      <c r="B205" t="str">
+        <v>/ˈask/</v>
+      </c>
+      <c r="C205" t="str">
+        <v>to seek information by posing a question</v>
+      </c>
+      <c r="D205" t="str">
+        <v>to make a request</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="str">
+        <v>aware</v>
+      </c>
+      <c r="B206" t="str">
+        <v>/ə-ˈwer/</v>
+      </c>
+      <c r="C206" t="str">
+        <v>having or showing understanding or knowledge : conscious</v>
+      </c>
+      <c r="D206" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="str">
+        <v>bad</v>
+      </c>
+      <c r="B207" t="str">
+        <v>/ˈbad/</v>
+      </c>
+      <c r="C207" t="str">
+        <v>not good : poor</v>
+      </c>
+      <c r="D207" t="str">
+        <v>not favorable</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="str">
+        <v>bags</v>
+      </c>
+      <c r="B208" t="str">
+        <v>/ˈbag/</v>
+      </c>
+      <c r="C208" t="str">
+        <v>a container made of flexible material (as paper or plastic)</v>
+      </c>
+      <c r="D208" t="str">
+        <v>purse, handbag</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="str">
+        <v>bake</v>
+      </c>
+      <c r="B209" t="str">
+        <v>/ˈbāk/</v>
+      </c>
+      <c r="C209" t="str">
+        <v>to cook or become cooked in a dry heat especially in an oven</v>
+      </c>
+      <c r="D209" t="str">
+        <v>to dry or harden by heat</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="str">
+        <v>bakes</v>
+      </c>
+      <c r="B210" t="str">
+        <v>/ˈbāk/</v>
+      </c>
+      <c r="C210" t="str">
+        <v>to cook or become cooked in a dry heat especially in an oven</v>
+      </c>
+      <c r="D210" t="str">
+        <v>to dry or harden by heat</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="str">
+        <v>beautiful</v>
+      </c>
+      <c r="B211" t="str">
+        <v>/ˈbyü-ti-fəl/</v>
+      </c>
+      <c r="C211" t="str">
+        <v>having qualities of beauty : giving pleasure to the mind or senses</v>
+      </c>
+      <c r="D211" t="str">
+        <v>very good : excellent</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="str">
+        <v>became</v>
+      </c>
+      <c r="B212" t="str">
+        <v>/bi-ˈkəm/</v>
+      </c>
+      <c r="C212" t="str">
+        <v>to come or grow to be</v>
+      </c>
+      <c r="D212" t="str">
+        <v>to be suitable to especially in a pleasing way</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="str">
+        <v>before</v>
+      </c>
+      <c r="B213" t="str">
+        <v>/bi-ˈfȯr/</v>
+      </c>
+      <c r="C213" t="str">
+        <v>at an earlier time</v>
+      </c>
+      <c r="D213" t="str">
+        <v>ahead</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="str">
+        <v>believing</v>
+      </c>
+      <c r="B214" t="str">
+        <v>/bə-ˈlēv/</v>
+      </c>
+      <c r="C214" t="str">
+        <v>to have faith or confidence in the existence or worth of</v>
+      </c>
+      <c r="D214" t="str">
+        <v>to accept as true</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="str">
+        <v>best</v>
+      </c>
+      <c r="B215" t="str">
+        <v>/ˈbest/</v>
+      </c>
+      <c r="C215" t="str">
+        <v>better than all others</v>
+      </c>
+      <c r="D215" t="str">
+        <v>most appropriate, useful, or helpful</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="str">
+        <v>bird</v>
+      </c>
+      <c r="B216" t="str">
+        <v>/ˈbərd/</v>
+      </c>
+      <c r="C216" t="str">
+        <v>an animal that lays eggs and has wings and a body covered with feathers</v>
+      </c>
+      <c r="D216" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="str">
+        <v>birthday</v>
+      </c>
+      <c r="B217" t="str">
+        <v>/ˈbərth-ˌdā/</v>
+      </c>
+      <c r="C217" t="str">
+        <v>the day or anniversary of someone's birth</v>
+      </c>
+      <c r="D217" t="str">
+        <v>a day of beginning</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="str">
+        <v>black</v>
+      </c>
+      <c r="B218" t="str">
+        <v>/ˈblak/</v>
+      </c>
+      <c r="C218" t="str">
+        <v>of the color of coal : colored black</v>
+      </c>
+      <c r="D218" t="str">
+        <v>very dark</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="str">
+        <v>both</v>
+      </c>
+      <c r="B219" t="str">
+        <v>/ˈbōth/</v>
+      </c>
+      <c r="C219" t="str">
+        <v>each one of two things or people : the two</v>
+      </c>
+      <c r="D219" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="str">
+        <v>bright</v>
+      </c>
+      <c r="B220" t="str">
+        <v>/ˈbrīt/</v>
+      </c>
+      <c r="C220" t="str">
+        <v>giving off or filled with much light</v>
+      </c>
+      <c r="D220" t="str">
+        <v>very clear or vivid in color</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="str">
+        <v>brings</v>
+      </c>
+      <c r="B221" t="str">
+        <v>/ˈbriŋ/</v>
+      </c>
+      <c r="C221" t="str">
+        <v>to cause to come by carrying or leading : take along</v>
+      </c>
+      <c r="D221" t="str">
+        <v>to cause to reach a certain state or take a certain action</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="str">
+        <v>brought</v>
+      </c>
+      <c r="B222" t="str">
+        <v/>
+      </c>
+      <c r="C222" t="str">
+        <v/>
+      </c>
+      <c r="D222" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="str">
+        <v>bus</v>
+      </c>
+      <c r="B223" t="str">
+        <v>/ˈbəs/</v>
+      </c>
+      <c r="C223" t="str">
+        <v>a large motor vehicle for carrying passengers</v>
+      </c>
+      <c r="D223" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="str">
+        <v>by</v>
+      </c>
+      <c r="B224" t="str">
+        <v>/bī/</v>
+      </c>
+      <c r="C224" t="str">
+        <v>close to : near</v>
+      </c>
+      <c r="D224" t="str">
+        <v>so as to go on</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="str">
+        <v>cake</v>
+      </c>
+      <c r="B225" t="str">
+        <v>/ˈkāk/</v>
+      </c>
+      <c r="C225" t="str">
+        <v>a baked food made from a sweet batter or dough</v>
+      </c>
+      <c r="D225" t="str">
+        <v>a usually flat round piece of food that is baked or fried</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="str">
+        <v>cart</v>
+      </c>
+      <c r="B226" t="str">
+        <v>/ˈkärt/</v>
+      </c>
+      <c r="C226" t="str">
+        <v>a heavy vehicle with two wheels usually drawn by horses and used for hauling</v>
+      </c>
+      <c r="D226" t="str">
+        <v>a light vehicle pushed or pulled by hand</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="str">
+        <v>clap</v>
+      </c>
+      <c r="B227" t="str">
+        <v>/ˈklap/</v>
+      </c>
+      <c r="C227" t="str">
+        <v>to hit (the palms of the hands) together usually more than once</v>
+      </c>
+      <c r="D227" t="str">
+        <v>to hit or touch with the open hand</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="str">
+        <v>come</v>
+      </c>
+      <c r="B228" t="str">
+        <v>/ˈkəm/</v>
+      </c>
+      <c r="C228" t="str">
+        <v>to move toward : approach</v>
+      </c>
+      <c r="D228" t="str">
+        <v>to go or travel to a place</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="str">
+        <v>crying</v>
+      </c>
+      <c r="B229" t="str">
+        <v>/ˈkrī/</v>
+      </c>
+      <c r="C229" t="str">
+        <v>to shed tears : weep</v>
+      </c>
+      <c r="D229" t="str">
+        <v>to make a loud call : shout, exclaim</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="str">
+        <v>deeper</v>
+      </c>
+      <c r="B230" t="str">
+        <v>/ˈdēp/</v>
+      </c>
+      <c r="C230" t="str">
+        <v>reaching far down below the surface</v>
+      </c>
+      <c r="D230" t="str">
+        <v>reaching far inward or back from the front or outer part</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="str">
+        <v>did</v>
+      </c>
+      <c r="B231" t="str">
+        <v/>
+      </c>
+      <c r="C231" t="str">
+        <v/>
+      </c>
+      <c r="D231" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="str">
+        <v>dino</v>
+      </c>
+      <c r="B232" t="str">
+        <v/>
+      </c>
+      <c r="C232" t="str">
+        <v/>
+      </c>
+      <c r="D232" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="str">
+        <v>do</v>
+      </c>
+      <c r="B233" t="str">
+        <v>/dü/</v>
+      </c>
+      <c r="C233" t="str">
+        <v>to cause (as an act or action) to happen : perform</v>
+      </c>
+      <c r="D233" t="str">
+        <v>act, behave</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="str">
+        <v>dying</v>
+      </c>
+      <c r="B234" t="str">
+        <v/>
+      </c>
+      <c r="C234" t="str">
+        <v/>
+      </c>
+      <c r="D234" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="str">
+        <v>earth</v>
+      </c>
+      <c r="B235" t="str">
+        <v>/ˈərth/</v>
+      </c>
+      <c r="C235" t="str">
+        <v>the planet that we live on</v>
+      </c>
+      <c r="D235" t="str">
+        <v>land as distinguished from sea and air</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="str">
+        <v>every</v>
+      </c>
+      <c r="B236" t="str">
+        <v>/ˈev-rē/</v>
+      </c>
+      <c r="C236" t="str">
+        <v>including each of a group or series without leaving out any</v>
+      </c>
+      <c r="D236" t="str">
+        <v>at regularly spaced times or distances</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="str">
+        <v>everybody</v>
+      </c>
+      <c r="B237" t="str">
+        <v>/ˈev-ri-ˌbə-dē/</v>
+      </c>
+      <c r="C237" t="str">
+        <v>every person</v>
+      </c>
+      <c r="D237" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="str">
+        <v>everyone</v>
+      </c>
+      <c r="B238" t="str">
+        <v>/ˈev-rē-wən/</v>
+      </c>
+      <c r="C238" t="str">
+        <v>every person</v>
+      </c>
+      <c r="D238" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="str">
+        <v>everywhere</v>
+      </c>
+      <c r="B239" t="str">
+        <v>/ˈev-rē-ˌhwer/</v>
+      </c>
+      <c r="C239" t="str">
+        <v>in or to every place</v>
+      </c>
+      <c r="D239" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="str">
+        <v>excited</v>
+      </c>
+      <c r="B240" t="str">
+        <v>/ik-ˈsī-təd/</v>
+      </c>
+      <c r="C240" t="str">
+        <v>very enthusiastic and eager</v>
+      </c>
+      <c r="D240" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="str">
+        <v>exclaimed</v>
+      </c>
+      <c r="B241" t="str">
+        <v>/ik-ˈsklām/</v>
+      </c>
+      <c r="C241" t="str">
+        <v>to speak or cry out suddenly or with strong feeling</v>
+      </c>
+      <c r="D241" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="str">
+        <v>face</v>
+      </c>
+      <c r="B242" t="str">
+        <v>/ˈfās/</v>
+      </c>
+      <c r="C242" t="str">
+        <v>the front part of the head</v>
+      </c>
+      <c r="D242" t="str">
+        <v>an expression of the face</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="str">
+        <v>familliar</v>
+      </c>
+      <c r="B243" t="str">
+        <v/>
+      </c>
+      <c r="C243" t="str">
+        <v/>
+      </c>
+      <c r="D243" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="str">
+        <v>few</v>
+      </c>
+      <c r="B244" t="str">
+        <v>/ˈfyü/</v>
+      </c>
+      <c r="C244" t="str">
+        <v>not many people or things</v>
+      </c>
+      <c r="D244" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="str">
+        <v>fight</v>
+      </c>
+      <c r="B245" t="str">
+        <v>/ˈfīt/</v>
+      </c>
+      <c r="C245" t="str">
+        <v>to struggle in battle or in physical combat</v>
+      </c>
+      <c r="D245" t="str">
+        <v>to argue angrily : quarrel</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="str">
+        <v>fish-full</v>
+      </c>
+      <c r="B246" t="str">
+        <v/>
+      </c>
+      <c r="C246" t="str">
+        <v/>
+      </c>
+      <c r="D246" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="str">
+        <v>food</v>
+      </c>
+      <c r="B247" t="str">
+        <v>/ˈfüd/</v>
+      </c>
+      <c r="C247" t="str">
+        <v>the material that people and animals eat : material containing carbohydrates, fats, proteins, and supplements (as minerals and vitamins) that is taken in by and used in the living body for growth and repair and as a source of energy for activities</v>
+      </c>
+      <c r="D247" t="str">
+        <v>inorganic substances (as nitrate and carbon dioxide) taken in by green plants and used to build organic nutrients</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="str">
+        <v>forest</v>
+      </c>
+      <c r="B248" t="str">
+        <v>/ˈfȯr-əst/</v>
+      </c>
+      <c r="C248" t="str">
+        <v>a growth of trees and underbrush covering a large area</v>
+      </c>
+      <c r="D248" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="str">
+        <v>found</v>
+      </c>
+      <c r="B249" t="str">
+        <v/>
+      </c>
+      <c r="C249" t="str">
+        <v/>
+      </c>
+      <c r="D249" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="str">
+        <v>friends</v>
+      </c>
+      <c r="B250" t="str">
+        <v>/ˈfrend/</v>
+      </c>
+      <c r="C250" t="str">
+        <v>a person who has a strong liking for and trust in another person</v>
+      </c>
+      <c r="D250" t="str">
+        <v>a person who is not an enemy</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="str">
+        <v>garbage</v>
+      </c>
+      <c r="B251" t="str">
+        <v>/ˈgär-bij/</v>
+      </c>
+      <c r="C251" t="str">
+        <v>material (as waste food) that has been thrown out</v>
+      </c>
+      <c r="D251" t="str">
+        <v>something that is worthless, useless, or untrue</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="str">
+        <v>gate</v>
+      </c>
+      <c r="B252" t="str">
+        <v>/ˈgāt/</v>
+      </c>
+      <c r="C252" t="str">
+        <v>an opening in a wall or fence</v>
+      </c>
+      <c r="D252" t="str">
+        <v>a part of a barrier (as a fence) that opens and closes like a door</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="str">
+        <v>gift</v>
+      </c>
+      <c r="B253" t="str">
+        <v>/ˈgift/</v>
+      </c>
+      <c r="C253" t="str">
+        <v>a special ability : talent</v>
+      </c>
+      <c r="D253" t="str">
+        <v>something given : present</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="str">
+        <v>give</v>
+      </c>
+      <c r="B254" t="str">
+        <v>/ˈgiv/</v>
+      </c>
+      <c r="C254" t="str">
+        <v>to hand over to be kept : present</v>
+      </c>
+      <c r="D254" t="str">
+        <v>to cause to have</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="str">
+        <v>grabbed</v>
+      </c>
+      <c r="B255" t="str">
+        <v>/ˈgrab/</v>
+      </c>
+      <c r="C255" t="str">
+        <v>to grasp or seize suddenly</v>
+      </c>
+      <c r="D255" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="str">
+        <v>grandmother</v>
+      </c>
+      <c r="B256" t="str">
+        <v>/ˈgrand-ˌmə-t͟hər/</v>
+      </c>
+      <c r="C256" t="str">
+        <v>the mother of someone's father or mother</v>
+      </c>
+      <c r="D256" t="str">
+        <v>a female ancestor</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="str">
+        <v>had</v>
+      </c>
+      <c r="B257" t="str">
+        <v/>
+      </c>
+      <c r="C257" t="str">
+        <v/>
+      </c>
+      <c r="D257" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="str">
+        <v>hands</v>
+      </c>
+      <c r="B258" t="str">
+        <v>/ˈhand/</v>
+      </c>
+      <c r="C258" t="str">
+        <v>the body part at the end of the human arm that includes the fingers and thumb</v>
+      </c>
+      <c r="D258" t="str">
+        <v>a bodily structure (as the hind foot of an ape) like the human hand in function or form</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="str">
+        <v>happy</v>
+      </c>
+      <c r="B259" t="str">
+        <v>/ˈha-pē/</v>
+      </c>
+      <c r="C259" t="str">
+        <v>feeling or showing pleasure : glad</v>
+      </c>
+      <c r="D259" t="str">
+        <v>enjoying a condition or situation : content</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="str">
+        <v>have</v>
+      </c>
+      <c r="B260" t="str">
+        <v>/ˈhav/</v>
+      </c>
+      <c r="C260" t="str">
+        <v>to hold or own</v>
+      </c>
+      <c r="D260" t="str">
+        <v>to possess as a characteristic</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="str">
+        <v>her</v>
+      </c>
+      <c r="B261" t="str">
+        <v>/ˈhər/</v>
+      </c>
+      <c r="C261" t="str">
+        <v>relating to or belonging to a certain woman, girl, or female animal</v>
+      </c>
+      <c r="D261" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="str">
+        <v>herself</v>
+      </c>
+      <c r="B262" t="str">
+        <v>/hər-ˈself/</v>
+      </c>
+      <c r="C262" t="str">
+        <v>her own self</v>
+      </c>
+      <c r="D262" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="str">
+        <v>his</v>
+      </c>
+      <c r="B263" t="str">
+        <v>/hiz/</v>
+      </c>
+      <c r="C263" t="str">
+        <v>relating to or belonging to a certain man, boy, or male animal</v>
+      </c>
+      <c r="D263" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="str">
+        <v>home</v>
+      </c>
+      <c r="B264" t="str">
+        <v>/ˈhōm/</v>
+      </c>
+      <c r="C264" t="str">
+        <v>the house or apartment where a person lives</v>
+      </c>
+      <c r="D264" t="str">
+        <v>the place where a person was born or grew up</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="str">
+        <v>house</v>
+      </c>
+      <c r="B265" t="str">
+        <v>/ˈhau̇s/</v>
+      </c>
+      <c r="C265" t="str">
+        <v>a place built for people to live in</v>
+      </c>
+      <c r="D265" t="str">
+        <v>something (as a nest or den) used by an animal for shelter</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="str">
+        <v>hub</v>
+      </c>
+      <c r="B266" t="str">
+        <v>/ˈhəb/</v>
+      </c>
+      <c r="C266" t="str">
+        <v>the center of a wheel, propeller, or fan</v>
+      </c>
+      <c r="D266" t="str">
+        <v>a center of activity</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="str">
+        <v>huge</v>
+      </c>
+      <c r="B267" t="str">
+        <v>/ˈhyüj/</v>
+      </c>
+      <c r="C267" t="str">
+        <v>great in size or degree : vast</v>
+      </c>
+      <c r="D267" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="str">
+        <v>hugged</v>
+      </c>
+      <c r="B268" t="str">
+        <v>/ˈhəg/</v>
+      </c>
+      <c r="C268" t="str">
+        <v>to clasp in the arms : embrace</v>
+      </c>
+      <c r="D268" t="str">
+        <v>to keep close to</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="str">
+        <v>hungry</v>
+      </c>
+      <c r="B269" t="str">
+        <v>/ˈhəŋ-grē/</v>
+      </c>
+      <c r="C269" t="str">
+        <v>feeling or showing hunger</v>
+      </c>
+      <c r="D269" t="str">
+        <v>having a strong desire</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="str">
+        <v>i</v>
+      </c>
+      <c r="B270" t="str">
+        <v>/ˈī/</v>
+      </c>
+      <c r="C270" t="str">
+        <v>the ninth letter of the English alphabet</v>
+      </c>
+      <c r="D270" t="str">
+        <v>the number one in Roman numerals</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="str">
+        <v>in</v>
+      </c>
+      <c r="B271" t="str">
+        <v>/ˈin/</v>
+      </c>
+      <c r="C271" t="str">
+        <v>located or positioned within</v>
+      </c>
+      <c r="D271" t="str">
+        <v>into</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="str">
+        <v xml:space="preserve">its </v>
+      </c>
+      <c r="B272" t="str">
+        <v>/ˈits/</v>
+      </c>
+      <c r="C272" t="str">
+        <v>relating to or belonging to it or itself</v>
+      </c>
+      <c r="D272" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="str">
+        <v>jake</v>
+      </c>
+      <c r="B273" t="str">
+        <v/>
+      </c>
+      <c r="C273" t="str">
+        <v/>
+      </c>
+      <c r="D273" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="str">
+        <v>joy</v>
+      </c>
+      <c r="B274" t="str">
+        <v>/ˈjȯi/</v>
+      </c>
+      <c r="C274" t="str">
+        <v>a feeling of pleasure or happiness that comes from success, good fortune, or a sense of well-being</v>
+      </c>
+      <c r="D274" t="str">
+        <v>something that gives pleasure or happiness</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="str">
+        <v>just</v>
+      </c>
+      <c r="B275" t="str">
+        <v>/ˈjəst/</v>
+      </c>
+      <c r="C275" t="str">
+        <v>being what is deserved</v>
+      </c>
+      <c r="D275" t="str">
+        <v>having a foundation in fact or reason : reasonable</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="str">
+        <v>kate</v>
+      </c>
+      <c r="B276" t="str">
+        <v/>
+      </c>
+      <c r="C276" t="str">
+        <v/>
+      </c>
+      <c r="D276" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="str">
+        <v>know</v>
+      </c>
+      <c r="B277" t="str">
+        <v>/ˈnō/</v>
+      </c>
+      <c r="C277" t="str">
+        <v>to recognize the identity of</v>
+      </c>
+      <c r="D277" t="str">
+        <v>to be aware of the truth of</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="str">
+        <v>leafy</v>
+      </c>
+      <c r="B278" t="str">
+        <v>/ˈlē-fē/</v>
+      </c>
+      <c r="C278" t="str">
+        <v>having, covered with, or resembling leaves</v>
+      </c>
+      <c r="D278" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="str">
+        <v>letter</v>
+      </c>
+      <c r="B279" t="str">
+        <v>/ˈle-tər/</v>
+      </c>
+      <c r="C279" t="str">
+        <v>one of the marks that are symbols for speech sounds in writing or print and that make up the alphabet</v>
+      </c>
+      <c r="D279" t="str">
+        <v>a written or printed communication (as one sent through the mail)</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="str">
+        <v>light</v>
+      </c>
+      <c r="B280" t="str">
+        <v>/ˈlīt/</v>
+      </c>
+      <c r="C280" t="str">
+        <v>the bright form of energy given off by something (as the sun) that makes it possible to see</v>
+      </c>
+      <c r="D280" t="str">
+        <v>a source (as a lamp) of light</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="str">
+        <v>little</v>
+      </c>
+      <c r="B281" t="str">
+        <v>/ˈli-tᵊl/</v>
+      </c>
+      <c r="C281" t="str">
+        <v>small in size</v>
+      </c>
+      <c r="D281" t="str">
+        <v>small in quantity</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="str">
+        <v>looked</v>
+      </c>
+      <c r="B282" t="str">
+        <v>/ˈlu̇k/</v>
+      </c>
+      <c r="C282" t="str">
+        <v>to use the power of vision : see</v>
+      </c>
+      <c r="D282" t="str">
+        <v>to direct the attention or eyes</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="str">
+        <v>love</v>
+      </c>
+      <c r="B283" t="str">
+        <v>/ˈləv/</v>
+      </c>
+      <c r="C283" t="str">
+        <v>strong and warm affection (as of a parent for a child)</v>
+      </c>
+      <c r="D283" t="str">
+        <v>a great liking</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="str">
+        <v>make</v>
+      </c>
+      <c r="B284" t="str">
+        <v>/ˈmāk/</v>
+      </c>
+      <c r="C284" t="str">
+        <v>to form or put together out of material or parts</v>
+      </c>
+      <c r="D284" t="str">
+        <v>to cause to exist or occur</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="str">
+        <v>man</v>
+      </c>
+      <c r="B285" t="str">
+        <v>/ˈman/</v>
+      </c>
+      <c r="C285" t="str">
+        <v>an adult male human being</v>
+      </c>
+      <c r="D285" t="str">
+        <v>a human being : person</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="str">
+        <v>market</v>
+      </c>
+      <c r="B286" t="str">
+        <v>/ˈmär-kət/</v>
+      </c>
+      <c r="C286" t="str">
+        <v>a public place where people gather to buy and sell things</v>
+      </c>
+      <c r="D286" t="str">
+        <v>a store where foods are sold to the public</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="str">
+        <v>might</v>
+      </c>
+      <c r="B287" t="str">
+        <v>/ˈmīt/</v>
+      </c>
+      <c r="C287" t="str">
+        <v>—used as a helping verb to show that something is possible but not likely</v>
+      </c>
+      <c r="D287" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="str">
+        <v>mother</v>
+      </c>
+      <c r="B288" t="str">
+        <v>/ˈmə-t͟hər/</v>
+      </c>
+      <c r="C288" t="str">
+        <v>a female parent</v>
+      </c>
+      <c r="D288" t="str">
+        <v>a nun in charge of a convent</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="str">
+        <v>mountains</v>
+      </c>
+      <c r="B289" t="str">
+        <v>/ˈmau̇n-tᵊn/</v>
+      </c>
+      <c r="C289" t="str">
+        <v>a raised area of land higher than a hill</v>
+      </c>
+      <c r="D289" t="str">
+        <v>a great mass or huge number</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="str">
+        <v>much</v>
+      </c>
+      <c r="B290" t="str">
+        <v>/ˈməch/</v>
+      </c>
+      <c r="C290" t="str">
+        <v>great in amount or extent</v>
+      </c>
+      <c r="D290" t="str">
+        <v>great in importance</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="str">
+        <v>my</v>
+      </c>
+      <c r="B291" t="str">
+        <v>/ˈmī/</v>
+      </c>
+      <c r="C291" t="str">
+        <v>belonging or relating to me or myself</v>
+      </c>
+      <c r="D291" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="str">
+        <v>name</v>
+      </c>
+      <c r="B292" t="str">
+        <v>/ˈnām/</v>
+      </c>
+      <c r="C292" t="str">
+        <v>a word or combination of words by which a person or thing is known</v>
+      </c>
+      <c r="D292" t="str">
+        <v>reputation</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="str">
+        <v>named</v>
+      </c>
+      <c r="B293" t="str">
+        <v/>
+      </c>
+      <c r="C293" t="str">
+        <v>to choose a word or words by which something will be known : give a name to</v>
+      </c>
+      <c r="D293" t="str">
+        <v>to refer to by the word by which a person or thing is known : call by name</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="str">
+        <v>needs</v>
+      </c>
+      <c r="B294" t="str">
+        <v>/ˈnēd/</v>
+      </c>
+      <c r="C294" t="str">
+        <v>to suffer from the lack of something important to life or health</v>
+      </c>
+      <c r="D294" t="str">
+        <v>to be necessary</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="str">
+        <v xml:space="preserve">nest </v>
+      </c>
+      <c r="B295" t="str">
+        <v>/ˈnest/</v>
+      </c>
+      <c r="C295" t="str">
+        <v>a shelter made by an animal and especially a bird for its eggs and young</v>
+      </c>
+      <c r="D295" t="str">
+        <v>a place where some animals live and usually lay eggs</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="str">
+        <v>never</v>
+      </c>
+      <c r="B296" t="str">
+        <v>/ˈne-vər/</v>
+      </c>
+      <c r="C296" t="str">
+        <v>not ever : at no time</v>
+      </c>
+      <c r="D296" t="str">
+        <v>not to any extent or in any way</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="str">
+        <v>night</v>
+      </c>
+      <c r="B297" t="str">
+        <v>/ˈnīt/</v>
+      </c>
+      <c r="C297" t="str">
+        <v>the time between dusk and dawn when there is no sunlight</v>
+      </c>
+      <c r="D297" t="str">
+        <v>the early part of the night : nightfall</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="str">
+        <v>not</v>
+      </c>
+      <c r="B298" t="str">
+        <v>/ˈnät/</v>
+      </c>
+      <c r="C298" t="str">
+        <v>—used to make a word or group of words negative</v>
+      </c>
+      <c r="D298" t="str">
+        <v>—used to stand for the negative of a group of words that comes before</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="str">
+        <v>once</v>
+      </c>
+      <c r="B299" t="str">
+        <v>/ˈwəns/</v>
+      </c>
+      <c r="C299" t="str">
+        <v>one time only</v>
+      </c>
+      <c r="D299" t="str">
+        <v>at some time in the past : formerly</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="str">
+        <v>only</v>
+      </c>
+      <c r="B300" t="str">
+        <v>/ˈōn-lē/</v>
+      </c>
+      <c r="C300" t="str">
+        <v>alone in or of a class or kind : sole</v>
+      </c>
+      <c r="D300" t="str">
+        <v>best without doubt</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="str">
+        <v>or</v>
+      </c>
+      <c r="B301" t="str">
+        <v>/ər/</v>
+      </c>
+      <c r="C301" t="str">
+        <v>—used between words or phrases that are choices</v>
+      </c>
+      <c r="D301" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="str">
+        <v>palm</v>
+      </c>
+      <c r="B302" t="str">
+        <v>/ˈpäm/</v>
+      </c>
+      <c r="C302" t="str">
+        <v>a tropical tree, shrub, or vine with a usually tall stem or trunk topped with large leaves that are shaped like feathers or fans</v>
+      </c>
+      <c r="D302" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="str">
+        <v>people</v>
+      </c>
+      <c r="B303" t="str">
+        <v>/ˈpē-pəl/</v>
+      </c>
+      <c r="C303" t="str">
+        <v>all persons considered together</v>
+      </c>
+      <c r="D303" t="str">
+        <v>a group of human beings who have something in common The word people is often used in compounds instead of persons.</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="str">
+        <v>pests</v>
+      </c>
+      <c r="B304" t="str">
+        <v>/ˈpest/</v>
+      </c>
+      <c r="C304" t="str">
+        <v>nuisance</v>
+      </c>
+      <c r="D304" t="str">
+        <v>a plant or animal that is harmful to humans or property</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="str">
+        <v>pinched</v>
+      </c>
+      <c r="B305" t="str">
+        <v>/ˈpinch/</v>
+      </c>
+      <c r="C305" t="str">
+        <v>to squeeze between the finger and thumb or between the jaws of an instrument</v>
+      </c>
+      <c r="D305" t="str">
+        <v>to squeeze painfully</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="str">
+        <v>plant's</v>
+      </c>
+      <c r="B306" t="str">
+        <v/>
+      </c>
+      <c r="C306" t="str">
+        <v/>
+      </c>
+      <c r="D306" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="str">
+        <v>pollution</v>
+      </c>
+      <c r="B307" t="str">
+        <v>/pə-ˈlü-shən/</v>
+      </c>
+      <c r="C307" t="str">
+        <v>the action of making something impure and often unsafe or unsuitable for use : the state of being polluted</v>
+      </c>
+      <c r="D307" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="str">
+        <v>put</v>
+      </c>
+      <c r="B308" t="str">
+        <v>/ˈpu̇t/</v>
+      </c>
+      <c r="C308" t="str">
+        <v>to place in or move into a particular position</v>
+      </c>
+      <c r="D308" t="str">
+        <v>to bring into a specified state or condition</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="str">
+        <v>really</v>
+      </c>
+      <c r="B309" t="str">
+        <v>/ˈrē-ə-lē/</v>
+      </c>
+      <c r="C309" t="str">
+        <v>in fact</v>
+      </c>
+      <c r="D309" t="str">
+        <v>without question</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="str">
+        <v>rests</v>
+      </c>
+      <c r="B310" t="str">
+        <v/>
+      </c>
+      <c r="C310" t="str">
+        <v>something that is left over : remainder</v>
+      </c>
+      <c r="D310" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="str">
+        <v>rivers</v>
+      </c>
+      <c r="B311" t="str">
+        <v>/ˈri-vər/</v>
+      </c>
+      <c r="C311" t="str">
+        <v>a natural stream of water larger than a brook or creek</v>
+      </c>
+      <c r="D311" t="str">
+        <v>a large stream or flow</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="str">
+        <v>rolled</v>
+      </c>
+      <c r="B312" t="str">
+        <v>/ˈrōl/</v>
+      </c>
+      <c r="C312" t="str">
+        <v>to move or cause to move by turning over and over on a surface</v>
+      </c>
+      <c r="D312" t="str">
+        <v>to shape or become shaped in rounded form</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="str">
+        <v>saw</v>
+      </c>
+      <c r="B313" t="str">
+        <v/>
+      </c>
+      <c r="C313" t="str">
+        <v/>
+      </c>
+      <c r="D313" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="str">
+        <v>say</v>
+      </c>
+      <c r="B314" t="str">
+        <v>/ˈsā/</v>
+      </c>
+      <c r="C314" t="str">
+        <v>to express in words</v>
+      </c>
+      <c r="D314" t="str">
+        <v>to state as an opinion or decision : declare</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="str">
+        <v>says</v>
+      </c>
+      <c r="B315" t="str">
+        <v>/ˈsā/</v>
+      </c>
+      <c r="C315" t="str">
+        <v>to express in words</v>
+      </c>
+      <c r="D315" t="str">
+        <v>to state as an opinion or decision : declare</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="str">
+        <v>scout</v>
+      </c>
+      <c r="B316" t="str">
+        <v>/ˈskau̇t/</v>
+      </c>
+      <c r="C316" t="str">
+        <v>to explore an area to find out information about it</v>
+      </c>
+      <c r="D316" t="str">
+        <v>to search an area for someone or something</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="str">
+        <v>seas</v>
+      </c>
+      <c r="B317" t="str">
+        <v>/ˈsē/</v>
+      </c>
+      <c r="C317" t="str">
+        <v>a body of salt water not as large as an ocean and often nearly surrounded by land</v>
+      </c>
+      <c r="D317" t="str">
+        <v>ocean</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="str">
+        <v>seeing</v>
+      </c>
+      <c r="B318" t="str">
+        <v>/ˈsē/</v>
+      </c>
+      <c r="C318" t="str">
+        <v>to have the power of sight</v>
+      </c>
+      <c r="D318" t="str">
+        <v>to view with the eyes</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="str">
+        <v>seemed</v>
+      </c>
+      <c r="B319" t="str">
+        <v>/ˈsēm/</v>
+      </c>
+      <c r="C319" t="str">
+        <v>to give the impression of being : appear</v>
+      </c>
+      <c r="D319" t="str">
+        <v>—used to make a statement less forceful or more polite</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="str">
+        <v>shed</v>
+      </c>
+      <c r="B320" t="str">
+        <v>/ˈshed/</v>
+      </c>
+      <c r="C320" t="str">
+        <v>to give off in drops</v>
+      </c>
+      <c r="D320" t="str">
+        <v>to get rid of</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="str">
+        <v>shop</v>
+      </c>
+      <c r="B321" t="str">
+        <v>/ˈshäp/</v>
+      </c>
+      <c r="C321" t="str">
+        <v>a place where goods are sold : a usually small store</v>
+      </c>
+      <c r="D321" t="str">
+        <v>a worker's place of business</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="str">
+        <v>sight</v>
+      </c>
+      <c r="B322" t="str">
+        <v>/ˈsīt/</v>
+      </c>
+      <c r="C322" t="str">
+        <v>the function, process, or power of seeing : the sense by which a person or animal becomes aware of the position, form, and color of objects</v>
+      </c>
+      <c r="D322" t="str">
+        <v>the act of seeing</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="str">
+        <v>skip</v>
+      </c>
+      <c r="B323" t="str">
+        <v>/ˈskip/</v>
+      </c>
+      <c r="C323" t="str">
+        <v>to move by taking short light steps and jumps</v>
+      </c>
+      <c r="D323" t="str">
+        <v>to pass over or omit an item, space, or step</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="str">
+        <v>slowly</v>
+      </c>
+      <c r="B324" t="str">
+        <v>/ˈslō/</v>
+      </c>
+      <c r="C324" t="str">
+        <v>moving, flowing, or going at less than the usual speed</v>
+      </c>
+      <c r="D324" t="str">
+        <v>taking more time than is expected or desired</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="str">
+        <v>smiled</v>
+      </c>
+      <c r="B325" t="str">
+        <v>/ˈsmīl/</v>
+      </c>
+      <c r="C325" t="str">
+        <v>make the corners of the mouth turn up in an expression of amusement or pleasure</v>
+      </c>
+      <c r="D325" t="str">
+        <v>to look with amusement or pleasure</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="str">
+        <v>smiles</v>
+      </c>
+      <c r="B326" t="str">
+        <v>/ˈsmīl/</v>
+      </c>
+      <c r="C326" t="str">
+        <v>make the corners of the mouth turn up in an expression of amusement or pleasure</v>
+      </c>
+      <c r="D326" t="str">
+        <v>to look with amusement or pleasure</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="str">
+        <v>so</v>
+      </c>
+      <c r="B327" t="str">
+        <v>/ˈsō/</v>
+      </c>
+      <c r="C327" t="str">
+        <v>in the way indicated</v>
+      </c>
+      <c r="D327" t="str">
+        <v>in the same way : also</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="str">
+        <v>spent</v>
+      </c>
+      <c r="B328" t="str">
+        <v>/ˈspent/</v>
+      </c>
+      <c r="C328" t="str">
+        <v>used up</v>
+      </c>
+      <c r="D328" t="str">
+        <v>drained of energy</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="str">
+        <v>started</v>
+      </c>
+      <c r="B329" t="str">
+        <v>/ˈstärt/</v>
+      </c>
+      <c r="C329" t="str">
+        <v>to begin an activity</v>
+      </c>
+      <c r="D329" t="str">
+        <v>to come or bring into being or action</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="str">
+        <v>stood</v>
+      </c>
+      <c r="B330" t="str">
+        <v/>
+      </c>
+      <c r="C330" t="str">
+        <v/>
+      </c>
+      <c r="D330" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="str">
+        <v>strong</v>
+      </c>
+      <c r="B331" t="str">
+        <v>/ˈstrȯŋ/</v>
+      </c>
+      <c r="C331" t="str">
+        <v>having great power in the muscles</v>
+      </c>
+      <c r="D331" t="str">
+        <v>healthy</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="str">
+        <v>swim</v>
+      </c>
+      <c r="B332" t="str">
+        <v>/ˈswim/</v>
+      </c>
+      <c r="C332" t="str">
+        <v>to move through or in water by moving arms, legs, fins, or tail</v>
+      </c>
+      <c r="D332" t="str">
+        <v>to cross by swimming</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="str">
+        <v>swing</v>
+      </c>
+      <c r="B333" t="str">
+        <v>/ˈswiŋ/</v>
+      </c>
+      <c r="C333" t="str">
+        <v>to move rapidly in a sweeping curve</v>
+      </c>
+      <c r="D333" t="str">
+        <v>to turn on a hinge or pivot</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="str">
+        <v>tall</v>
+      </c>
+      <c r="B334" t="str">
+        <v>/ˈtȯl/</v>
+      </c>
+      <c r="C334" t="str">
+        <v>having unusually great height</v>
+      </c>
+      <c r="D334" t="str">
+        <v>of a stated height</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="str">
+        <v>taller</v>
+      </c>
+      <c r="B335" t="str">
+        <v>/ˈtȯl/</v>
+      </c>
+      <c r="C335" t="str">
+        <v>having unusually great height</v>
+      </c>
+      <c r="D335" t="str">
+        <v>of a stated height</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="str">
+        <v>tears</v>
+      </c>
+      <c r="B336" t="str">
+        <v>/ˈtir/</v>
+      </c>
+      <c r="C336" t="str">
+        <v>a drop of the salty liquid that moistens the eyes and the inner eyelids and that flows from the eyes when someone is crying</v>
+      </c>
+      <c r="D336" t="str">
+        <v>an act of crying</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="str">
+        <v>teary-eyed</v>
+      </c>
+      <c r="B337" t="str">
+        <v/>
+      </c>
+      <c r="C337" t="str">
+        <v/>
+      </c>
+      <c r="D337" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="str">
+        <v>tell</v>
+      </c>
+      <c r="B338" t="str">
+        <v>/ˈtel/</v>
+      </c>
+      <c r="C338" t="str">
+        <v>to let a person know something : to give information to</v>
+      </c>
+      <c r="D338" t="str">
+        <v>order</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="str">
+        <v>than</v>
+      </c>
+      <c r="B339" t="str">
+        <v>/t͟hən/</v>
+      </c>
+      <c r="C339" t="str">
+        <v>when compared to the way in which, the extent to which, or the degree to which</v>
+      </c>
+      <c r="D339" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="str">
+        <v>thank</v>
+      </c>
+      <c r="B340" t="str">
+        <v>/ˈthaŋk/</v>
+      </c>
+      <c r="C340" t="str">
+        <v>to express gratitude to</v>
+      </c>
+      <c r="D340" t="str">
+        <v>to hold responsible</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="str">
+        <v>that</v>
+      </c>
+      <c r="B341" t="str">
+        <v>/ˈt͟hat/</v>
+      </c>
+      <c r="C341" t="str">
+        <v>the person or thing seen, mentioned, or understood</v>
+      </c>
+      <c r="D341" t="str">
+        <v>the time, action, or event mentioned</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="str">
+        <v>their</v>
+      </c>
+      <c r="B342" t="str">
+        <v>/t͟hər/</v>
+      </c>
+      <c r="C342" t="str">
+        <v>of or relating to them or themselves especially as owners or as agents or objects of an action</v>
+      </c>
+      <c r="D342" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="str">
+        <v>then</v>
+      </c>
+      <c r="B343" t="str">
+        <v>/ˈt͟hen/</v>
+      </c>
+      <c r="C343" t="str">
+        <v>at that time</v>
+      </c>
+      <c r="D343" t="str">
+        <v>soon after that : next</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="str">
+        <v>these</v>
+      </c>
+      <c r="B344" t="str">
+        <v/>
+      </c>
+      <c r="C344" t="str">
+        <v/>
+      </c>
+      <c r="D344" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="str">
+        <v>this</v>
+      </c>
+      <c r="B345" t="str">
+        <v>/ˈt͟his/</v>
+      </c>
+      <c r="C345" t="str">
+        <v>the one nearer</v>
+      </c>
+      <c r="D345" t="str">
+        <v>the person, thing, or idea that is present or near in place, time, or thought or that has just been mentioned</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="str">
+        <v>time</v>
+      </c>
+      <c r="B346" t="str">
+        <v>/ˈtīm/</v>
+      </c>
+      <c r="C346" t="str">
+        <v>a period during which an action, process, or condition exists or continues</v>
+      </c>
+      <c r="D346" t="str">
+        <v>a point or period when something occurs : occasion</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="str">
+        <v>tina</v>
+      </c>
+      <c r="B347" t="str">
+        <v/>
+      </c>
+      <c r="C347" t="str">
+        <v/>
+      </c>
+      <c r="D347" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="str">
+        <v>together</v>
+      </c>
+      <c r="B348" t="str">
+        <v>/tə-ˈge-t͟hər/</v>
+      </c>
+      <c r="C348" t="str">
+        <v>in or into one group, body, or place</v>
+      </c>
+      <c r="D348" t="str">
+        <v>in touch or in partnership with</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="str">
+        <v>toward</v>
+      </c>
+      <c r="B349" t="str">
+        <v>/ˈtō-ərd/</v>
+      </c>
+      <c r="C349" t="str">
+        <v>in the direction of</v>
+      </c>
+      <c r="D349" t="str">
+        <v>along a course leading to</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="str">
+        <v>tree</v>
+      </c>
+      <c r="B350" t="str">
+        <v>/ˈtrē/</v>
+      </c>
+      <c r="C350" t="str">
+        <v>a long-lived woody plant that has a single usually tall main stem with few or no branches on its lower part</v>
+      </c>
+      <c r="D350" t="str">
+        <v>a plant of treelike form</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="str">
+        <v>trees</v>
+      </c>
+      <c r="B351" t="str">
+        <v>/ˈtrē/</v>
+      </c>
+      <c r="C351" t="str">
+        <v>a long-lived woody plant that has a single usually tall main stem with few or no branches on its lower part</v>
+      </c>
+      <c r="D351" t="str">
+        <v>a plant of treelike form</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="str">
+        <v>turtle</v>
+      </c>
+      <c r="B352" t="str">
+        <v>/ˈtər-tᵊl/</v>
+      </c>
+      <c r="C352" t="str">
+        <v>a reptile that lives on land, in water, or both and has a toothless horny beak and a shell of bony plates which covers the body and into which the head, legs, and tail can usually be drawn</v>
+      </c>
+      <c r="D352" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="str">
+        <v>ugly</v>
+      </c>
+      <c r="B353" t="str">
+        <v>/ˈə-glē/</v>
+      </c>
+      <c r="C353" t="str">
+        <v>unpleasant to look at : not attractive</v>
+      </c>
+      <c r="D353" t="str">
+        <v>offensive</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="str">
+        <v>up</v>
+      </c>
+      <c r="B354" t="str">
+        <v>/ˈəp/</v>
+      </c>
+      <c r="C354" t="str">
+        <v>in or to a high or higher place or position</v>
+      </c>
+      <c r="D354" t="str">
+        <v>in or into a vertical position</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="str">
+        <v>upon</v>
+      </c>
+      <c r="B355" t="str">
+        <v>/ə-ˈpȯn/</v>
+      </c>
+      <c r="C355" t="str">
+        <v>on</v>
+      </c>
+      <c r="D355" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="str">
+        <v>us</v>
+      </c>
+      <c r="B356" t="str">
+        <v>/əs/</v>
+      </c>
+      <c r="C356" t="str">
+        <v/>
+      </c>
+      <c r="D356" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="str">
+        <v>valentine</v>
+      </c>
+      <c r="B357" t="str">
+        <v>/ˈva-lən-ˌtīn/</v>
+      </c>
+      <c r="C357" t="str">
+        <v>a greeting card or gift sent or given on Valentine's Day</v>
+      </c>
+      <c r="D357" t="str">
+        <v>a sweetheart given something as a sign of affection on Valentine's Day</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="str">
+        <v>very</v>
+      </c>
+      <c r="B358" t="str">
+        <v>/ˈver-ē/</v>
+      </c>
+      <c r="C358" t="str">
+        <v>to a great degree : extremely</v>
+      </c>
+      <c r="D358" t="str">
+        <v>in actual fact : truly</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="str">
+        <v>want</v>
+      </c>
+      <c r="B359" t="str">
+        <v>/ˈwȯnt/</v>
+      </c>
+      <c r="C359" t="str">
+        <v>to desire, wish, or long for something</v>
+      </c>
+      <c r="D359" t="str">
+        <v>to feel or suffer the need of something</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="str">
+        <v>way</v>
+      </c>
+      <c r="B360" t="str">
+        <v>/ˈwā/</v>
+      </c>
+      <c r="C360" t="str">
+        <v>the manner in which something is done or happens</v>
+      </c>
+      <c r="D360" t="str">
+        <v>the course traveled from one place to another : route</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="str">
+        <v>went</v>
+      </c>
+      <c r="B361" t="str">
+        <v/>
+      </c>
+      <c r="C361" t="str">
+        <v/>
+      </c>
+      <c r="D361" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="str">
+        <v>were</v>
+      </c>
+      <c r="B362" t="str">
+        <v/>
+      </c>
+      <c r="C362" t="str">
+        <v/>
+      </c>
+      <c r="D362" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="str">
+        <v>west</v>
+      </c>
+      <c r="B363" t="str">
+        <v>/ˈwest/</v>
+      </c>
+      <c r="C363" t="str">
+        <v>to or toward the direction of sunset</v>
+      </c>
+      <c r="D363" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="str">
+        <v>what</v>
+      </c>
+      <c r="B364" t="str">
+        <v>/ˈhwät/</v>
+      </c>
+      <c r="C364" t="str">
+        <v>which thing or things</v>
+      </c>
+      <c r="D364" t="str">
+        <v>which sort of thing or person</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="str">
+        <v>whatever</v>
+      </c>
+      <c r="B365" t="str">
+        <v>/hwät-ˈe-vər/</v>
+      </c>
+      <c r="C365" t="str">
+        <v>anything or everything that</v>
+      </c>
+      <c r="D365" t="str">
+        <v>no matter what</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="str">
+        <v>who</v>
+      </c>
+      <c r="B366" t="str">
+        <v>/ˈhü/</v>
+      </c>
+      <c r="C366" t="str">
+        <v>what or which person or people</v>
+      </c>
+      <c r="D366" t="str">
+        <v>—used to stand for a person or people at the beginning of a clause</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="str">
+        <v>why</v>
+      </c>
+      <c r="B367" t="str">
+        <v>/ˈhwī/</v>
+      </c>
+      <c r="C367" t="str">
+        <v>for what cause or reason</v>
+      </c>
+      <c r="D367" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="str">
+        <v>won't</v>
+      </c>
+      <c r="B368" t="str">
+        <v>/ˈwōnt/</v>
+      </c>
+      <c r="C368" t="str">
+        <v>will not</v>
+      </c>
+      <c r="D368" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="str">
+        <v>wrap</v>
+      </c>
+      <c r="B369" t="str">
+        <v>/ˈrap/</v>
+      </c>
+      <c r="C369" t="str">
+        <v>to cover by winding or folding</v>
+      </c>
+      <c r="D369" t="str">
+        <v>to enclose in a package</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="str">
+        <v>wreath</v>
+      </c>
+      <c r="B370" t="str">
+        <v>/ˈrēth/</v>
+      </c>
+      <c r="C370" t="str">
+        <v>something twisted or woven into a circular shape</v>
+      </c>
+      <c r="D370" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="str">
+        <v>wren</v>
+      </c>
+      <c r="B371" t="str">
+        <v>/ˈren/</v>
+      </c>
+      <c r="C371" t="str">
+        <v>a small brown songbird with a short tail that points upward</v>
+      </c>
+      <c r="D371" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="str">
+        <v>wrinkle</v>
+      </c>
+      <c r="B372" t="str">
+        <v>/ˈriŋ-kəl/</v>
+      </c>
+      <c r="C372" t="str">
+        <v>a crease or small fold (as in the skin or in cloth)</v>
+      </c>
+      <c r="D372" t="str">
+        <v>a clever notion or trick</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="str">
+        <v>write</v>
+      </c>
+      <c r="B373" t="str">
+        <v>/ˈrīt/</v>
+      </c>
+      <c r="C373" t="str">
+        <v>to form letters or words with pen or pencil</v>
+      </c>
+      <c r="D373" t="str">
+        <v>to form the letters or the words of (as on paper)</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="str">
+        <v>wrong</v>
+      </c>
+      <c r="B374" t="str">
+        <v>/ˈrȯŋ/</v>
+      </c>
+      <c r="C374" t="str">
+        <v>not the one wanted or intended</v>
+      </c>
+      <c r="D374" t="str">
+        <v>not correct or true : false</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="str">
+        <v>yes</v>
+      </c>
+      <c r="B375" t="str">
+        <v>/ˈyes/</v>
+      </c>
+      <c r="C375" t="str">
+        <v>—used to express agreement in answer to a question, request, or offer or with an earlier statement</v>
+      </c>
+      <c r="D375" t="str">
+        <v>—used to introduce a phrase with greater emphasis or clearness</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="str">
+        <v>you</v>
+      </c>
+      <c r="B376" t="str">
+        <v>/ˈyü/</v>
+      </c>
+      <c r="C376" t="str">
+        <v>the person, thing, or group these words are spoken or written to</v>
+      </c>
+      <c r="D376" t="str">
+        <v>anyone at all</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D197"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D376"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fixed stt and ai feedback
</commit_message>
<xml_diff>
--- a/mobile/ipa.xlsx
+++ b/mobile/ipa.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D376"/>
+  <dimension ref="A1:D413"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5663,9 +5663,527 @@
         <v>anyone at all</v>
       </c>
     </row>
+    <row r="377">
+      <c r="A377" t="str">
+        <v>crow</v>
+      </c>
+      <c r="B377" t="str">
+        <v>/ˈkrō/</v>
+      </c>
+      <c r="C377" t="str">
+        <v>a glossy black bird that has a harsh cry</v>
+      </c>
+      <c r="D377" t="str">
+        <v>a member of a tribe of Indigenous people of Montana</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="str">
+        <v>picked</v>
+      </c>
+      <c r="B378" t="str">
+        <v>/ˈpik/</v>
+      </c>
+      <c r="C378" t="str">
+        <v>to gather one by one</v>
+      </c>
+      <c r="D378" t="str">
+        <v>to remove bit by bit</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="str">
+        <v>some</v>
+      </c>
+      <c r="B379" t="str">
+        <v>/ˈsəm/</v>
+      </c>
+      <c r="C379" t="str">
+        <v>not known, named, or specified</v>
+      </c>
+      <c r="D379" t="str">
+        <v>being one, a part, or an unspecified number of something</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="str">
+        <v>stones</v>
+      </c>
+      <c r="B380" t="str">
+        <v>/ˈstōn/</v>
+      </c>
+      <c r="C380" t="str">
+        <v>earth or mineral matter hardened in a mass : rock</v>
+      </c>
+      <c r="D380" t="str">
+        <v>a piece of rock coarser than gravel</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="str">
+        <v>ted</v>
+      </c>
+      <c r="B381" t="str">
+        <v/>
+      </c>
+      <c r="C381" t="str">
+        <v/>
+      </c>
+      <c r="D381" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="str">
+        <v>seed</v>
+      </c>
+      <c r="B382" t="str">
+        <v>/ˈsēd/</v>
+      </c>
+      <c r="C382" t="str">
+        <v>a tiny developing plant that is enclosed in a protective coat usually along with a supply of food and that is able to develop under suitable conditions into a plant like the one that produced it</v>
+      </c>
+      <c r="D382" t="str">
+        <v>a small structure (as a spore or a tiny dry fruit) other than a true seed by which a plant reproduces itself</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="str">
+        <v>grain</v>
+      </c>
+      <c r="B383" t="str">
+        <v>/ˈgrān/</v>
+      </c>
+      <c r="C383" t="str">
+        <v>the edible seed or seeds of some grasses (as wheat, corn, or oats) or a few other plants (as buckwheat)</v>
+      </c>
+      <c r="D383" t="str">
+        <v>plants that produce grain</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="str">
+        <v>are</v>
+      </c>
+      <c r="B384" t="str">
+        <v/>
+      </c>
+      <c r="C384" t="str">
+        <v/>
+      </c>
+      <c r="D384" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="str">
+        <v>man</v>
+      </c>
+      <c r="B385" t="str">
+        <v>/ˈman/</v>
+      </c>
+      <c r="C385" t="str">
+        <v>an adult male human being</v>
+      </c>
+      <c r="D385" t="str">
+        <v>a human being : person</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="str">
+        <v>road</v>
+      </c>
+      <c r="B386" t="str">
+        <v>/ˈrōd/</v>
+      </c>
+      <c r="C386" t="str">
+        <v>a hard flat surface for vehicles, persons, and animals to travel on</v>
+      </c>
+      <c r="D386" t="str">
+        <v>a way to achieve something</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="str">
+        <v>meal</v>
+      </c>
+      <c r="B387" t="str">
+        <v>/ˈmēl/</v>
+      </c>
+      <c r="C387" t="str">
+        <v>the food eaten or prepared for eating at one time</v>
+      </c>
+      <c r="D387" t="str">
+        <v>the act or time of eating</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="str">
+        <v>alex</v>
+      </c>
+      <c r="B388" t="str">
+        <v/>
+      </c>
+      <c r="C388" t="str">
+        <v/>
+      </c>
+      <c r="D388" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="str">
+        <v>ball</v>
+      </c>
+      <c r="B389" t="str">
+        <v>/ˈbȯl/</v>
+      </c>
+      <c r="C389" t="str">
+        <v>something round or roundish</v>
+      </c>
+      <c r="D389" t="str">
+        <v>a round or roundish object used in a game or sport</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="str">
+        <v>gray</v>
+      </c>
+      <c r="B390" t="str">
+        <v/>
+      </c>
+      <c r="C390" t="str">
+        <v>of a color that is a blend of black and white</v>
+      </c>
+      <c r="D390" t="str">
+        <v>having gray hair</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="str">
+        <v>bunny</v>
+      </c>
+      <c r="B391" t="str">
+        <v>/ˈbə-nē/</v>
+      </c>
+      <c r="C391" t="str">
+        <v>rabbit</v>
+      </c>
+      <c r="D391" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="str">
+        <v>crabs</v>
+      </c>
+      <c r="B392" t="str">
+        <v>/ˈkrab/</v>
+      </c>
+      <c r="C392" t="str">
+        <v>a sea animal that is a crustacean related to the lobsters and has a short broad flat shell and a front pair of legs with small claws</v>
+      </c>
+      <c r="D392" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="str">
+        <v>have</v>
+      </c>
+      <c r="B393" t="str">
+        <v>/ˈhav/</v>
+      </c>
+      <c r="C393" t="str">
+        <v>to hold or own</v>
+      </c>
+      <c r="D393" t="str">
+        <v>to possess as a characteristic</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="str">
+        <v>hard</v>
+      </c>
+      <c r="B394" t="str">
+        <v>/ˈhärd/</v>
+      </c>
+      <c r="C394" t="str">
+        <v>not easily cut, pierced, or divided : not soft</v>
+      </c>
+      <c r="D394" t="str">
+        <v>difficult to do or to understand</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="str">
+        <v>shells</v>
+      </c>
+      <c r="B395" t="str">
+        <v>/ˈshel/</v>
+      </c>
+      <c r="C395" t="str">
+        <v>a stiff hard covering of an animal (as a turtle, oyster, or crab)</v>
+      </c>
+      <c r="D395" t="str">
+        <v>the tough outer covering of an egg</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="str">
+        <v>wash</v>
+      </c>
+      <c r="B396" t="str">
+        <v>/ˈwȯsh/</v>
+      </c>
+      <c r="C396" t="str">
+        <v>to cleanse with water and usually a cleaning agent (as soap)</v>
+      </c>
+      <c r="D396" t="str">
+        <v>to wet completely with liquid</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="str">
+        <v>iron</v>
+      </c>
+      <c r="B397" t="str">
+        <v>/ˈī-ərn/</v>
+      </c>
+      <c r="C397" t="str">
+        <v>a heavy silvery white metallic chemical element that rusts easily, is strongly attracted by magnets, occurs in meteorites and combined in minerals, and is necessary for transporting oxygen in the blood</v>
+      </c>
+      <c r="D397" t="str">
+        <v>a device that is heated and used for making cloth smooth</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="str">
+        <v>dress</v>
+      </c>
+      <c r="B398" t="str">
+        <v>/ˈdres/</v>
+      </c>
+      <c r="C398" t="str">
+        <v>to put clothes on</v>
+      </c>
+      <c r="D398" t="str">
+        <v>to put on clothes in a particular way</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="str">
+        <v>dog</v>
+      </c>
+      <c r="B399" t="str">
+        <v>/ˈdȯg/</v>
+      </c>
+      <c r="C399" t="str">
+        <v>a domestic animal that eats meat and is closely related to the wolves</v>
+      </c>
+      <c r="D399" t="str">
+        <v>any of the group of mammals (as wolves, foxes, and jackals) to which the domestic dog belongs</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="str">
+        <v>has</v>
+      </c>
+      <c r="B400" t="str">
+        <v/>
+      </c>
+      <c r="C400" t="str">
+        <v/>
+      </c>
+      <c r="D400" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="str">
+        <v>collar</v>
+      </c>
+      <c r="B401" t="str">
+        <v>/ˈkä-lər/</v>
+      </c>
+      <c r="C401" t="str">
+        <v>the part of a piece of clothing that fits around a person's neck</v>
+      </c>
+      <c r="D401" t="str">
+        <v>a band of material worn around an animal's neck</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="str">
+        <v>jumps</v>
+      </c>
+      <c r="B402" t="str">
+        <v>/ˈjəmp/</v>
+      </c>
+      <c r="C402" t="str">
+        <v>to spring into the air : leap</v>
+      </c>
+      <c r="D402" t="str">
+        <v>to pass over or cause to pass over with or as if with a leap</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="str">
+        <v>mat</v>
+      </c>
+      <c r="B403" t="str">
+        <v>/ˈmat/</v>
+      </c>
+      <c r="C403" t="str">
+        <v>a piece of material used as a floor or seat covering or in front of a door to wipe the shoes on</v>
+      </c>
+      <c r="D403" t="str">
+        <v>a decorative piece of material used under dishes or vases</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="str">
+        <v>hug</v>
+      </c>
+      <c r="B404" t="str">
+        <v>/ˈhəg/</v>
+      </c>
+      <c r="C404" t="str">
+        <v>to clasp in the arms : embrace</v>
+      </c>
+      <c r="D404" t="str">
+        <v>to keep close to</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="str">
+        <v>animals</v>
+      </c>
+      <c r="B405" t="str">
+        <v>/ˈa-nə-məl/</v>
+      </c>
+      <c r="C405" t="str">
+        <v>any member of the kingdom of living things (as earthworms, crabs, birds, and people) that differ from plants typically in being able to move about, in not having cell walls made of cellulose, and in depending on plants and other animals as sources of food</v>
+      </c>
+      <c r="D405" t="str">
+        <v>any of the animals lower than humans in the natural order</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="str">
+        <v>felt</v>
+      </c>
+      <c r="B406" t="str">
+        <v>/ˈfelt/</v>
+      </c>
+      <c r="C406" t="str">
+        <v>a soft heavy cloth made by rolling and pressing fibers together</v>
+      </c>
+      <c r="D406" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="str">
+        <v>rug</v>
+      </c>
+      <c r="B407" t="str">
+        <v>/ˈrəg/</v>
+      </c>
+      <c r="C407" t="str">
+        <v>a piece of thick heavy fabric usually with a nap or pile used especially as a floor covering</v>
+      </c>
+      <c r="D407" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="str">
+        <v>dusty</v>
+      </c>
+      <c r="B408" t="str">
+        <v>/ˈdə-stē/</v>
+      </c>
+      <c r="C408" t="str">
+        <v>filled or covered with dust</v>
+      </c>
+      <c r="D408" t="str">
+        <v>resembling dust</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="str">
+        <v>read</v>
+      </c>
+      <c r="B409" t="str">
+        <v>/ˈrēd/</v>
+      </c>
+      <c r="C409" t="str">
+        <v>to understand language through written symbols for speech sounds</v>
+      </c>
+      <c r="D409" t="str">
+        <v>to speak aloud written or printed words</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="str">
+        <v>library</v>
+      </c>
+      <c r="B410" t="str">
+        <v>/ˈlī-ˌbrer-ē/</v>
+      </c>
+      <c r="C410" t="str">
+        <v>a place where literary or reference materials (as books, manuscripts, recordings, or films) are kept for use but are not for sale</v>
+      </c>
+      <c r="D410" t="str">
+        <v>a collection of literary or reference materials</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="str">
+        <v>books</v>
+      </c>
+      <c r="B411" t="str">
+        <v>/ˈbu̇k/</v>
+      </c>
+      <c r="C411" t="str">
+        <v>a set of sheets of paper bound together</v>
+      </c>
+      <c r="D411" t="str">
+        <v>a long written work</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="str">
+        <v>learn</v>
+      </c>
+      <c r="B412" t="str">
+        <v>/ˈlərn/</v>
+      </c>
+      <c r="C412" t="str">
+        <v>to get knowledge of or skill in by study, instruction, or experience</v>
+      </c>
+      <c r="D412" t="str">
+        <v>memorize</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="str">
+        <v>things</v>
+      </c>
+      <c r="B413" t="str">
+        <v>/ˈthiŋ/</v>
+      </c>
+      <c r="C413" t="str">
+        <v>an act or matter that is or is to be done</v>
+      </c>
+      <c r="D413" t="str">
+        <v>something that exists and can be talked about</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D376"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D413"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>